<commit_message>
xlsx added floor and room
</commit_message>
<xml_diff>
--- a/src/data/exhibition-imports/template/artist-submission-template.xlsx
+++ b/src/data/exhibition-imports/template/artist-submission-template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Study/Projects/Cutare/cutare-gallery/src/data/exhibition-imports/template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7474A573-6AF6-2740-9A5A-F5E1541E808B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43FEE4A0-BAC7-DC40-B409-4B44E5264E27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Artist" sheetId="1" r:id="rId1"/>
@@ -19,8 +19,66 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Eliza Balica</author>
+  </authors>
+  <commentList>
+    <comment ref="D7" authorId="0" shapeId="0" xr:uid="{5D19A723-DD33-3E4F-AC47-8E1871DAE85D}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Se completeaza de catre curator</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E7" authorId="0" shapeId="0" xr:uid="{EC8AFA6F-DF5D-BC40-BE74-A8E77B827617}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="14"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>Se completează de către curator</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="14"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="10">
   <si>
     <t>nume artist</t>
   </si>
@@ -44,13 +102,19 @@
   </si>
   <si>
     <t>descriere</t>
+  </si>
+  <si>
+    <t>etaj</t>
+  </si>
+  <si>
+    <t>sala</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -69,6 +133,32 @@
       <color rgb="FF000000"/>
       <name val="Bell MT"/>
       <family val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -91,7 +181,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -114,23 +204,55 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB0B0B0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB0B0B0"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFB0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFB0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -138,6 +260,24 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -479,82 +619,80 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C16"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="24" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="39.83203125" style="4" customWidth="1"/>
-    <col min="2" max="2" width="20" style="3" customWidth="1"/>
-    <col min="3" max="3" width="60" style="3" customWidth="1"/>
-    <col min="4" max="16384" width="8.83203125" style="3"/>
+    <col min="1" max="1" width="39.83203125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="20" style="1" customWidth="1"/>
+    <col min="3" max="3" width="60" style="1" customWidth="1"/>
+    <col min="4" max="4" width="16.1640625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="15.1640625" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+      <c r="B1" s="9"/>
+      <c r="C1" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+      <c r="B2" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
+      <c r="B3" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="5" t="s">
+      <c r="B4" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B7" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C7" s="8" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D7" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
         <v>1</v>
       </c>
@@ -564,92 +702,163 @@
       <c r="C8" s="7" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="B14" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="B15" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="B16" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="C16" s="7" t="s">
+      <c r="D8" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E17" s="4" t="s">
         <v>1</v>
       </c>
     </row>
@@ -661,5 +870,6 @@
     <mergeCell ref="B4:C4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>